<commit_message>
Update in monitoring history and lit review. A csv with a set of indicators for ELC is added, after a literature review.
</commit_message>
<xml_diff>
--- a/notes/Literature_Review.xlsx
+++ b/notes/Literature_Review.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="energy use" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="LC indicators" sheetId="2" state="visible" r:id="rId3"/>
-    <sheet name="demand modeling in the south" sheetId="3" state="visible" r:id="rId4"/>
-    <sheet name="methods" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="LC papers" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="LC indicators" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="demand modeling in the south" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="methods" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="185">
   <si>
     <t xml:space="preserve">Author(s)</t>
   </si>
@@ -223,157 +224,208 @@
     <t xml:space="preserve">To provide a comprensive approach of energy use through the Capabilities perspective of Amartya Sen.</t>
   </si>
   <si>
+    <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Main purpose of the study</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approach (modelling, real data measuring)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simulation tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temporal level/timestep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sally Köhler, Ruben Rongstock, Martin Hein, Ursula Eicker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Similarity measures and comparison methods for residential electricity load profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy &amp; Buildings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baden-Württemberg, Germany</t>
+  </si>
+  <si>
+    <t xml:space="preserve">households</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To present an approach that addresses the issue of assessing the similarity or representativeness of electricity load profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Measuring and real data modelling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLPG, SimStadt, SynPro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 minute</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matthew Li, David Allinson, Miaomiao He</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seasonal variation in household electricity demand: A comparison of monitored and synthetic daily load profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stefano Mandelli, Marco Merlo, Emanuela Colombo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Novel procedure to formulate load profiles for off-grid rural areas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy for Sustainable Development</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Omotola Adeoye, Catalina Spataru</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelling and forecasting hourly electricity demand in West African countries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied Energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. Sandels, J. Widén, L. Nordström</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forecasting household consumer electricity load profiles with a combined physical and behavioral approach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ángela Herraiz-Cañete, David Ribó-Pérez, Paula Bastida-Molina, Tomás Gómez-Navarro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forecasting energy demand in isolated rural communities: A comparison between deterministic and stochastic approaches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El Salvador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">households, community services, IGA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serge Guefano, Jean Gaston Tamba, Tchitile Emmanuel Wilfried Azong, Louis Monkam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Forecast of electricity consumption in the Cameroonian residential sector by Grey and vector autoregressive models</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energy </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cristina Dominguez, Kristina Orehounig, Jan Carmeliet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estimating hourly lighting load profiles of rural households in East Africa applying a data-driven characterization of occupant behavior and lighting devices ownership</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Development Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joakim Wide ́, Magdalena Lundh, Iana Vassileva, Erik Dahlquist, Kajsa Ellega ̊, Ewa Wa ̈ ckelga ̊ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Constructing load profiles for household electricity and hot water from time-use data—Modelling approach and validation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elias Hartvigsson, Erik O. Ahlgren </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comparison of load profiles in a mini-grid: Assessment of performance metrics using measured and interview-based data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luca Lorenzoni, Paolo Cherubini, Davide Fioriti, Davide Poli, Andrea Micangeli, Romano Giglioli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classification and modeling of load profiles of isolated mini-grids in developing countries: A data-driven approach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yue Zhu and Jovica V. Milanovic ́</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automatic Identification of Power System Load  Models Based on Field Measurements</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IEEE Transactions on Power Systems</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Courtney Blodgetta, Peter Dauenhauerb, Henry Louiec, Lauren Kickhama</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accuracy of energy-use surveys in predicting rural mini-grid user consumption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J. Dickert and P. Schegner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Time Series Probabilistic Synthetic Load  Curve Model for Residential Customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2011 IEEE Trondheim PowerTech</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Angreine Kewo, Pinrolinvic D. K. Manembu and Per Sieverts Nielsen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Rigorous Standalone Literature Review of Residential Electricity Load Profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sandhya Patidar∗, David P. Jenkins and Sophie A. Simpson</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stochastic modelling techniques for generating synthetic energy demand profiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">International Journal of Energy and Statistics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicators Used</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicator type (magnitud and intensity, shape and efficiency, temporal and timing, variability and statistical, etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicator formula</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Limitations / Challenges Noted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual consumption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fractal dimension (FD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RMSE (Root Mean Square Error) of Load Duration Curves (LDCs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NRMSE (Normalized Root Mean Square Error) of LDCs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Violin Plots</t>
+  </si>
+  <si>
     <t xml:space="preserve">Load Curve Type</t>
   </si>
   <si>
     <t xml:space="preserve">Validation Purpose</t>
   </si>
   <si>
-    <t xml:space="preserve">Indicators Used</t>
-  </si>
-  <si>
     <t xml:space="preserve">Indicator Formula / Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Limitations / Challenges Noted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sally Köhler, Ruben Rongstock, Martin Hein, Ursula Eicker</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Similarity measures and comparison methods for residential electricity load profiles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energy &amp; Buildings</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baden-Württemberg, Germany</t>
-  </si>
-  <si>
-    <t xml:space="preserve">households</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Matthew Li, David Allinson, Miaomiao He</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seasonal variation in household electricity demand: A comparison of monitored and synthetic daily load profiles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stefano Mandelli, Marco Merlo, Emanuela Colombo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Novel procedure to formulate load profiles for off-grid rural areas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energy for Sustainable Development</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Omotola Adeoye, Catalina Spataru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelling and forecasting hourly electricity demand in West African countries</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Applied Energy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C. Sandels, J. Widén, L. Nordström</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forecasting household consumer electricity load profiles with a combined physical and behavioral approach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sweden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ángela Herraiz-Cañete, David Ribó-Pérez, Paula Bastida-Molina, Tomás Gómez-Navarro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forecasting energy demand in isolated rural communities: A comparison between deterministic and stochastic approaches</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El Salvador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">households, community services, IGA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serge Guefano, Jean Gaston Tamba, Tchitile Emmanuel Wilfried Azong, Louis Monkam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Forecast of electricity consumption in the Cameroonian residential sector by Grey and vector autoregressive models</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energy </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cristina Dominguez, Kristina Orehounig, Jan Carmeliet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estimating hourly lighting load profiles of rural households in East Africa applying a data-driven characterization of occupant behavior and lighting devices ownership</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Development Engineering</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Joakim Wide ́, Magdalena Lundh, Iana Vassileva, Erik Dahlquist, Kajsa Ellega ̊, Ewa Wa ̈ ckelga ̊ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Constructing load profiles for household electricity and hot water from time-use data—Modelling approach and validation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elias Hartvigsson, Erik O. Ahlgren </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comparison of load profiles in a mini-grid: Assessment of performance metrics using measured and interview-based data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luca Lorenzoni, Paolo Cherubini, Davide Fioriti, Davide Poli, Andrea Micangeli, Romano Giglioli</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Classification and modeling of load profiles of isolated mini-grids in developing countries: A data-driven approach</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yue Zhu and Jovica V. Milanovic ́</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Automatic Identification of Power System Load  Models Based on Field Measurements</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IEEE Transactions on Power Systems</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Courtney Blodgetta, Peter Dauenhauerb, Henry Louiec, Lauren Kickhama</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Accuracy of energy-use surveys in predicting rural mini-grid user consumption</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J. Dickert and P. Schegner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Time Series Probabilistic Synthetic Load  Curve Model for Residential Customers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2011 IEEE Trondheim PowerTech</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Angreine Kewo, Pinrolinvic D. K. Manembu and Per Sieverts Nielsen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Rigorous Standalone Literature Review of Residential Electricity Load Profiles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Energies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sandhya Patidar∗, David P. Jenkins and Sophie A. Simpson</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stochastic modelling techniques for generating synthetic energy demand profiles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">International Journal of Energy and Statistics</t>
   </si>
   <si>
     <t xml:space="preserve">Subhes C. Bhattacharyya, Govinda R. Timilsina</t>
@@ -536,13 +588,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -565,7 +616,13 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -617,7 +674,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -638,12 +695,20 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -754,7 +819,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="108.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
         <v>21</v>
       </c>
@@ -786,7 +851,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="68.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
         <v>29</v>
       </c>
@@ -879,7 +944,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="121.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="108.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>53</v>
       </c>
@@ -911,7 +976,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="55.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
         <v>61</v>
       </c>
@@ -939,8 +1004,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -950,85 +1015,74 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P17"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="25.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="26.9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21.61"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17.42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="19.62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="23.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17.98"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="24.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="23.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="30.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="20.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="29.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="32.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34.18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="38.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="21.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="31.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="33.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="9" style="0" width="20.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="29.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="32.41"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+    <row r="1" customFormat="false" ht="53.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="J1" s="1" t="s">
+      <c r="H1" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="I1" s="6" t="s">
         <v>69</v>
       </c>
+      <c r="J1" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="K1" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="L1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="P1" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="0" t="n">
+    <row r="2" customFormat="false" ht="55.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="0" t="n">
         <v>2022</v>
-      </c>
-      <c r="C2" s="0" t="s">
-        <v>72</v>
       </c>
       <c r="D2" s="0" t="s">
         <v>73</v>
@@ -1039,236 +1093,296 @@
       <c r="F2" s="0" t="s">
         <v>75</v>
       </c>
+      <c r="G2" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="G3" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="B3" s="0" t="n">
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>86</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="E6" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="0" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E7" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="F7" s="0" t="s">
+        <v>94</v>
+      </c>
+      <c r="G7" s="0" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>97</v>
+      </c>
+      <c r="E8" s="0" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="0" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>2009</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" s="0" t="n">
         <v>2018</v>
       </c>
-      <c r="C3" s="0" t="s">
-        <v>77</v>
-      </c>
-      <c r="D3" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" s="0" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="B4" s="0" t="n">
+      <c r="D11" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="0" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="0" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>2011</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>117</v>
+      </c>
+      <c r="E16" s="0" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="0" t="s">
+        <v>119</v>
+      </c>
+      <c r="C17" s="0" t="n">
         <v>2016</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="0" t="n">
-        <v>2019</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="B6" s="0" t="n">
-        <v>2014</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>85</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>83</v>
-      </c>
-      <c r="E6" s="0" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" s="0" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="0" t="n">
-        <v>2022</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>80</v>
-      </c>
-      <c r="E7" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="F7" s="0" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>91</v>
-      </c>
-      <c r="B8" s="0" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="B9" s="0" t="n">
-        <v>2021</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="B10" s="0" t="n">
-        <v>2009</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="B11" s="0" t="n">
-        <v>2018</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="B12" s="0" t="n">
-        <v>2020</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="B13" s="0" t="n">
-        <v>2018</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>104</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>106</v>
-      </c>
-      <c r="B14" s="0" t="n">
-        <v>2017</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>108</v>
-      </c>
-      <c r="B15" s="0" t="n">
-        <v>2011</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>109</v>
-      </c>
-      <c r="D15" s="0" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>111</v>
-      </c>
-      <c r="B16" s="0" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" s="0" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
-        <v>114</v>
-      </c>
-      <c r="B17" s="0" t="n">
-        <v>2016</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>115</v>
-      </c>
       <c r="D17" s="0" t="s">
-        <v>116</v>
-      </c>
-      <c r="F17" s="0" t="s">
-        <v>75</v>
+        <v>120</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="G17" s="0" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1287,8 +1401,76 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="39.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="17.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.31"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>130</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPágina &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:P2"/>
-  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.171875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.86"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26.87"/>
@@ -1318,25 +1500,25 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>66</v>
+        <v>131</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>67</v>
+        <v>132</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>68</v>
+        <v>122</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>69</v>
+        <v>133</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>10</v>
@@ -1348,15 +1530,15 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>2010</v>
       </c>
       <c r="C2" s="0" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>
@@ -1364,19 +1546,19 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L1048576"/>
-  <sheetFormatPr defaultColWidth="9.15234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="29.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28.76"/>
@@ -1410,46 +1592,46 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="I1" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="K1" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H1" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="B2" s="0" t="n">
         <v>2018</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E2" s="0" t="s">
         <v>24</v>
       </c>
       <c r="F2" s="0" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="H2" s="0" t="s">
         <v>63</v>
@@ -1461,186 +1643,185 @@
         <v>63</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="188.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>2019</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="162.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="B4" s="0" t="n">
         <v>2020</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="D4" s="0" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="E4" s="0" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="162.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>2016</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="B6" s="0" t="n">
         <v>2017</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>47</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="F6" s="0" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="H6" s="0" t="s">
         <v>58</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="K6" s="0" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="68.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="B7" s="0" t="n">
         <v>2017</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>47</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="H7" s="0" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="K7" s="0" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+        <v>184</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>